<commit_message>
histogramas - erro em tempestade
</commit_message>
<xml_diff>
--- a/resultados_kp.xlsx
+++ b/resultados_kp.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,6 +456,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Kp parcial (02h até 05h)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Classificacao</t>
         </is>
       </c>
@@ -467,7 +472,10 @@
       <c r="B2" t="n">
         <v>3.3</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -480,7 +488,10 @@
       <c r="B3" t="n">
         <v>3</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -493,7 +504,10 @@
       <c r="B4" t="n">
         <v>4</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
@@ -506,7 +520,10 @@
       <c r="B5" t="n">
         <v>2.3</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -519,7 +536,10 @@
       <c r="B6" t="n">
         <v>3</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -532,7 +552,10 @@
       <c r="B7" t="n">
         <v>2.7</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -545,7 +568,10 @@
       <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -558,7 +584,10 @@
       <c r="B9" t="n">
         <v>5</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Tempestade</t>
         </is>
@@ -571,7 +600,10 @@
       <c r="B10" t="n">
         <v>5.7</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>Tempestade</t>
         </is>
@@ -584,7 +616,10 @@
       <c r="B11" t="n">
         <v>4.3</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
@@ -597,7 +632,10 @@
       <c r="B12" t="n">
         <v>4.3</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
@@ -610,7 +648,10 @@
       <c r="B13" t="n">
         <v>4</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
@@ -623,7 +664,10 @@
       <c r="B14" t="n">
         <v>3.3</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -636,7 +680,10 @@
       <c r="B15" t="n">
         <v>3.3</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -649,7 +696,10 @@
       <c r="B16" t="n">
         <v>2.3</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -662,7 +712,10 @@
       <c r="B17" t="n">
         <v>1.7</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -675,7 +728,10 @@
       <c r="B18" t="n">
         <v>1.7</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -688,7 +744,10 @@
       <c r="B19" t="n">
         <v>3</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -701,7 +760,10 @@
       <c r="B20" t="n">
         <v>4.7</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
@@ -714,7 +776,10 @@
       <c r="B21" t="n">
         <v>4</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
@@ -727,7 +792,10 @@
       <c r="B22" t="n">
         <v>2.7</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D22" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -740,7 +808,10 @@
       <c r="B23" t="n">
         <v>3</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -753,7 +824,10 @@
       <c r="B24" t="n">
         <v>2</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -766,7 +840,10 @@
       <c r="B25" t="n">
         <v>1.7</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -779,7 +856,10 @@
       <c r="B26" t="n">
         <v>3</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -792,7 +872,10 @@
       <c r="B27" t="n">
         <v>2.7</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="D27" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -805,7 +888,10 @@
       <c r="B28" t="n">
         <v>2.7</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D28" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -818,7 +904,10 @@
       <c r="B29" t="n">
         <v>2</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -831,7 +920,10 @@
       <c r="B30" t="n">
         <v>2</v>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -844,7 +936,10 @@
       <c r="B31" t="n">
         <v>2.3</v>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>
@@ -857,7 +952,10 @@
       <c r="B32" t="n">
         <v>2.3</v>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t>Calmo</t>
         </is>

</xml_diff>